<commit_message>
Excel: cronograma detallado en hoja 2
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YFGBiKFSRgr65g49Ta8xpm
</commit_message>
<xml_diff>
--- a/projects/2026-10-02_diplomado_neuro_urgencias_kine/Programa_detallado_jornada_neurologia_USS_actualizado.xlsx
+++ b/projects/2026-10-02_diplomado_neuro_urgencias_kine/Programa_detallado_jornada_neurologia_USS_actualizado.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Programa" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos generales" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cronograma detallado" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos generales" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -628,6 +629,546 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.4" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="100" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="45" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Bloque</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Horario y duración</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Actividad</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Tipo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="21" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>08:30–08:40 (10 min)</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Bienvenida, reglas de la sesión online, encuesta diagnóstica en vivo</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Interacción</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="21" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>08:40–08:50 (10 min)</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Caso gancho: paciente somnolienta con signos de herniación (votación: Glasgow y primera acción)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="21" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>08:50–09:05 (15 min)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Micro-clase 1: Glasgow, pupilas, patrón respiratorio, signos de HTIC y herniación</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="21" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>09:05–09:20 (15 min)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Micro-clase 2: coma estructural vs metabólico; banderas rojas de cefalea y vértigo central</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="36" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>09:20–09:45 (25 min)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>PRÁCTICA 1: puntuar Glasgow y pupilas en videos de pacientes simulados (votación) + salas pequeñas con 2 casos y SBAR de 30 s</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Práctica</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="21" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>09:45–09:50 (5 min)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Cierre: mensajes clave y pregunta de foro 1</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="21" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>10:00–10:10 (10 min)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Caso gancho: ACV en urgencia, ¿qué hora anoto y qué hago en 5 minutos?</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="21" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>10:10–10:30 (20 min)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Micro-clase 1: isquemia vs hemorragia, BE-FAST, reloj del ACV, conceptos de reperfusión</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="36" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>10:30–10:45 (15 min)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Micro-clase 2: primeros minutos (ABCDE), oxígeno, glicemia, ayuno hasta tamizaje de deglución, rol kinésico</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="36" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>10:45–11:15 (30 min)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>PRÁCTICA 2: caso ramificado en salas pequeñas con 3 puntos de decisión (reconocer / tiempo y vía aérea / reporte y traslado)</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Práctica</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="21" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>11:15–11:20 (5 min)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Cierre y pregunta de foro 2</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="21" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>11:30–11:40 (10 min)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Caso gancho: crisis tónico-clónica en sala de espera (¿qué hago y qué no hago?)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Caso</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="21" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>11:40–12:00 (20 min)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Micro-clase 1: qué es una crisis y qué no (mimics), primeros pasos y regla de 5 minutos</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="21" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>12:00–12:15 (15 min)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Micro-clase 2: estatus epiléptico, escalonamiento de fármacos, vía aérea y ventilación</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>12:15–12:50 (35 min)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>PRÁCTICA 3: simulación en salas con roles (líder, vía aérea, medicación, registro) y checklist de desempeño</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Práctica</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="21" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>12:50–13:00 (10 min)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Debriefing y pregunta de foro 3</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="21" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>13:00–14:00 (60 min)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Receso. Almuerzo.</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Receso</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="21" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>14:00–14:05 (5 min)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Reactivación: pregunta de votación de repaso</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Interacción</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="21" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>14:05–14:25 (20 min)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Micro-clase 1: meningitis/encefalitis, HSA y hemorragia intracerebral, HTIC</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="21" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>14:25–14:45 (20 min)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Micro-clase 2: neuroventilación (metas de SpO2 y PaCO2, aspiración, posición, errores a evitar)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Teoría</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="36" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>14:45–15:15 (30 min)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>PRÁCTICA 4: caso integrador escalonado (HSA con GCS 8): reconocer, asegurar vía aérea, ventilar, trasladar</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Práctica</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="21" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>15:15–15:20 (5 min)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Cierre del módulo, evaluación formativa, pregunta de foro 4</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Cierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>330 minutos de actividad; 120 minutos de práctica en vivo (36%).</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>